<commit_message>
feat: production-ready voice calling pipeline
- Pre-recorded greeting plays first, Gemini Live S2S connects during playback
- Prompt/RAG/greeting/language fully frontend-configurable (DB-driven, no hardcode)
- Agent name follows saved prompt (removed hardcoded persona anchors)
- Removed legacy villa scripts from runtime turn injections
- Telugu-first + multilingual mirroring, transcription on gemini-3.1-flash-lite
- Campaign orchestration: dialing-at-claim, parallel dials, repeat schedules
- Source/broker filter, KPI real 7-day trends, Voice & Language config card
- Hermes watchdog + DEBUGGING_REPORT.xlsx (64/64 tests)
</commit_message>
<xml_diff>
--- a/DEBUGGING_REPORT.xlsx
+++ b/DEBUGGING_REPORT.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -101,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,6 +127,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -546,9 +550,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -632,6 +633,66 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>Gemini prepayment credits depleted - top up in AI Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Round 2 (PostgreSQL migration + 3-agent audit)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>27 bugs found &amp; fixed; full suite 51/51 green on PostgreSQL; app boots with 151 routes; weekly ZIP + migration + DNC verified end-to-end</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Round 3 (frontend funnel + Vobiz plug-and-play + digital 2-concurrency)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>5 items fixed; suite 55/55 green; funnel+Vobiz card deployed to VPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Round 4 (KPI honesty + Vobiz extras/webhooks + funnel nav + prompt chain + campaign enforcement + Hermes watchdog)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>6 items fixed; suite 61/61 green; watchdog cron live on VPS every 5 min with TTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Round 5 (live dialing status + broker source filter + chart layout + real KPI trends + watchdog runner)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5 items fixed; suite 63/63 green; V7 deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Round 6 (pre-recorded greeting plays + Gemini S2S + Telugu primary + transcription fixed)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>5 items fixed; suite 64/64 green; V8 deployed; language=te-IN mirror=ON</t>
         </is>
       </c>
     </row>
@@ -650,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1414,6 +1475,2456 @@
       <c r="J15" s="8" t="inlineStr">
         <is>
           <t>VPS endpoints 200, role-scoped</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Database / Core</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>App was PostgreSQL-only with NO local/dev fallback: default DSN host 'postgres' never resolves outside docker, so local dev, CI and the whole test suite crashed at startup (RuntimeError: could not translate host name 'postgres'). Plan requires 'PostgreSQL (production) and SQLite (development fallback)'.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>core/db.py default_dsn() hard-coded host='postgres' (docker network alias) as the default for every environment; docker-compose never passed PGHOST explicitly.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>default_dsn() now defaults to localhost; docker-compose sets PGHOST=postgres + PG* creds explicitly for the container. Tests now run against a dedicated technopoliss_test Postgres DB (tests/helpers.py) via the real production storage path.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>backend/core/db.py, docker-compose.yml, backend/tests/helpers.py, backend/tests/test_orchestration.py, backend/tests/test_audit_fixes_smoke.py, backend/tests/test_digital_excel_ingest.py</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Core / Lead Memory</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>lead_memory.get_memory crashed on Postgres: positional fallback row[2] grabbed last_interaction_at (float) instead of summary (index 1) because DictRow is not sqlite3.Row — every memory read raised AttributeError: 'float' object has no attribute 'strip'. Memory-aware dials (plan Phase 5) were broken on the real DB.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Positional index fallback assumed row[2]=summary; SELECT order is facts_json(0), summary(1), last_interaction_at(2), version(3). Only masked on Postgres shim (DictRow).</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Rewrote get_memory with name-first accessor + correct positional fallback (summary=1, version=3).</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>backend/core/lead_memory.py</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>WhatsApp / Orchestration</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>live_job_executor.execute_whatsapp_job wrote datetime('now') (-&gt; now(), a timestamptz) into leads.whatsapp_sent_at REAL column -&gt; DatatypeMismatch on Postgres; the bare except: pass swallowed it, so the brochure send was recorded as never-sent (whatsapp_sent stayed 0) and duplicate brochures could be sent.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>REAL (epoch) timestamp column assigned a timestamptz via the SQL translation layer; also `import time` was missing so the replacement raised NameError, also swallowed.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Store epoch seconds (time.time()) as a parameter like every other REAL timestamp column; added the missing import.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>backend/core/live_job_executor.py</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Orchestration / Concurrency</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>workflow_queue.claim_next was not atomic under concurrency: SELECT then UPDATE in READ COMMITTED let two workers both pass the lead-lock NOT EXISTS check and claim the same job (or two jobs of one lead) — duplicate dials (plan Phase 4 SKIP LOCKED requirement violated).</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Two-statement claim without FOR UPDATE / SKIP LOCKED; lead row never locked.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Postgres path now selects with FOR UPDATE OF j, l SKIP LOCKED inside the claim transaction and claims with a conditional UPDATE (rowcount check); added _unclaim + number_resolver for atomic claim+line assignment. Added 5 concurrency tests.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>backend/core/workflow_queue.py, backend/core/orchestration_dispatcher.py</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Orchestration / Routing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Callbacks rang from the WRONG originating line: dispatcher peeked lead source with a separate SELECT, then claimed whatever job won the race — a digital callback could ring from P1/P2 cold line.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Line chosen before claim; not resolved from the actually-claimed job.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Added _job_lead_source + number_resolver passed into claim_next so the callback line (P1/P2 cold, P3 digital) is resolved from the claimed job inside the same transaction; dispatcher re-checks line lock/cooldown post-claim.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>backend/core/orchestration_dispatcher.py, backend/core/workflow_queue.py</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Orchestration</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PRIORITY dict missing JobType.SITE_VISIT_RESCHEDULE -&gt; KeyError crashed any site-visit reschedule at scheduling time, breaking the reschedule lifecycle.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>New job type added to enum but not to the priority table.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Added SITE_VISIT_RESCHEDULE: 4 to PRIORITY + regression test (every JobType covered).</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>backend/core/orchestration_service.py, backend/tests/test_audit_fixes_smoke.py</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MCP Server</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>get_lead_status crashed (AttributeError: str has no .get) because leads.extra is a JSON string in the DB; create_lead only inserted a row and never enqueued a fresh_call job — the MCP tools were effectively dead for the pipeline (plan objective 1.2).</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Extra read as dict; no job enqueued on create.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>_lead_extra_dict() tolerates dict or JSON string; _lead_sandbox() derives sandbox from column &gt; stage; create_lead now normalizes phone (E.164), persists budget/location/property_type into extra, enqueues fresh_call on the correct pool; trigger_manual_call checks operator dnc_list + do_not_contact register.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>backend/mcp_server.py</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>API / DND Compliance</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>create_callback (api/routes/callbacks.py) had no DNC enforcement — an operator could schedule a callback for an opted-out number (plan 1.4/4.3 compliance gap).</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Missing do_not_contact lookup before scheduling.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>create_callback now returns HTTP 409 'number is on the do-not-contact list' before scheduling.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>backend/api/routes/callbacks.py</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Orchestration / Dashboard</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>leads.sandbox column never updated by the event engine: failed calls never moved to SB2, callbacks never returned to SB1, interested leads never entered SB3 — dashboard sandbox views were wrong.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Event-to-job functions mutated lifecycle_status but not the sandbox column.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>_set_sandbox() helper wired into failed_call-&gt;SB2, schedule_callback-&gt;SB1, interested/whatsapp_package_sent-&gt;SB3; sandbox_for_stage(CALLBACK_REQUESTED) corrected to SB1 per plan flowchart. Added 4 sandbox-flow tests.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>backend/core/orchestration_service.py, backend/core/workflow_models.py, backend/tests/test_audit_fixes_smoke.py</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Voice / TTS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>gemini_tts.py used httpx.Optional[...] (httpx has no Optional attr) — pyflakes undefined names; latent import-time failure under type evaluation.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Invalid attribute access in annotations.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Replaced with Optional[httpx.AsyncClient] / Optional[httpx.Response] using typing.Optional.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>backend/services/gemini_tts.py</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Voice / Routes</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>web_voice.py /ws/voice-test called handle_browser_voice_ws which was never imported -&gt; NameError 500 on the browser voice test path (plan Section 4 manual test).</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Missing import.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Added from services.browser_voice_bridge import handle_browser_voice_ws.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>backend/api/routes/web_voice.py</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Voice / Routes</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>factory.py sandbox routes referenced create_agent/list_agents/etc. (undefined) -&gt; NameError on every /api/factory route (now correctly unmounted legacy; imports fixed so it parses).</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Missing imports from services.sandbox_manager.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Added the full sandbox_manager import set.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>backend/api/routes/factory.py</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>API / Routes</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>console_api.py virtual-meet endpoints called undefined extract_role(request) -&gt; NameError; virtual meet capture/reschedule could never be read.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Helper never defined in the module.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Added module-level extract_role (query param &gt; X-User-Role/X-Role header &gt; sales_1).</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>backend/api/routes/console_api.py</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DNC / Compliance</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>core/dnc.py used SQLite-only INSERT OR IGNORE into a private dnc_list table while the queue/dispatcher check do_not_contact — operator opt-outs were silently never recorded (TRAI/DND broken) and the two registers diverged.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>dnc.py predated the do_not_contact canonical table; INSERT OR IGNORE invalid on Postgres (swallowed by except).</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Rewrote dnc.py against the canonical do_not_contact(normalized_phone) table with ON CONFLICT DO UPDATE; add_to_dnc and opt_out now share one register; is_phone_blocked checks it (suffix + exact). Verified add/check/opt-out round trip on Postgres.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>backend/core/dnc.py</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Voice / Dialer</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>_process_single_lead (orchestration dial leg) had no DNC guard — an opt-out landing between job creation and execution would still be dialed.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Guard existed in campaign sub-workers but not the orchestration entry point.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Added is_phone_blocked check before marking dialing; returns dnc_blocked outcome without dialing.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>backend/core/worker.py</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Voice / Live Session</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>live_session.py: _activity_end_nudge_seq read/incremented in a nested Gemini handler without nonlocal -&gt; UnboundLocalError ('referenced before assignment') during activity-end nudges.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Missing nonlocal declaration for the enclosing-scope counter.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Added _activity_end_nudge_seq to the pump_gemini_to_queue nonlocal list.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>backend/services/vobiz_bridge/live_session.py</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Voice / Opening</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>build_opening_line ignored row_data entirely — every call got the static greeting even when the lead name/company was available.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Interpolation helpers existed but were unused.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Interpolate name + company via the existing helpers (fallback stays packaged line).</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>backend/core/opening_line.py</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ops / Weekly ZIP</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>weekly_zip_archive.py used a trailing 7-day window at runtime and never pruned originals — a Monday 6 AM run captured the current week instead of the PRIOR calendar week (plan Phase 7 violated).</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>mtime &gt;= now-7d window; no prune step.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Prior-calendar-week [Mon, Mon) bounds in Asia/Kolkata; prunes archived originals after a successful zip; dry_run flag; verified end-to-end with a temp recordings dir (zip contains only prior-week files).</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>backend/scripts/weekly_zip_archive.py</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Callbacks / Scheduler</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>callback_schedule.resolve_callback_epoch relative branch ('in 10 minutes') never shifted into the 11:00-19:30 IST window — a 7:35 PM callback was scheduled inside quiet hours (plan Phase 3).</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Relative targets computed as now+delta with no window slide.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Added _slide_into_working_hours: before-day -&gt; 11:00 same day, after 19:30 -&gt; next day 11:00; applied to relative + fallback branches; absolute times untouched. Verified 19:25+10min -&gt; next day 11:00.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>backend/services/callback_schedule.py</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>WhatsApp / Blue Loop</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>WhatsApp 'not interested again' was never handled: _classify_inbound_reply returned ('','') so the Blue Loop never reached terminal LOST/DNC (plan Phase 6).</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Not-interested phrases filtered out before classification.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Returns ('not_interested','whatsapp'); process_campaign_whatsapp_reply now calls orchestration opt_out (lead -&gt; opted_out/LOST, jobs cancelled, do_not_contact row) and publishes lead_updated.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>backend/services/whatsapp_leads.py</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>WhatsApp / Direct Booking</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Direct-booking bypass (willing-to-visit -&gt; Site Visit + cancel nudges) only ran AFTER a successful Gemini call — with no API key or on API failure the lead was never transitioned (plan Phase 6 bypass broken).</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Keyword logic inside the Gemini success path only.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Deterministic _detect_site_visit_intent + async _apply_site_visit_bypass run BEFORE Gemini (negation-aware); cancels whatsapp_followup_24h + interested_followup jobs; verified.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>backend/services/whatsapp_conversation.py</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>WhatsApp / Webhook</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Meta webhook had no idempotency on wa_message_id — retried deliveries caused duplicate lead updates + duplicate AI replies.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>No dedup tracking.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Thread-safe bounded LRU _MessageIdCache keyed on wa_message_id; seen ids short-circuit with dedup:true. Ingest exceptions now mark ignored so the AI reply step is skipped.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>backend/api/routes/whatsapp.py</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>WhatsApp / Workflow</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>On INTERESTED only a greeting text was sent; the brochure depended solely on the durable whatsapp_package job — a down/backlogged job loop meant no brochure (plan Phase 6 'WhatsApp Immediate Brochure').</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Brochure deferred to the job executor only.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>send_full_package also called inline on the INTERESTED transition (guarded try/except), keeping the durable job as source of truth.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>backend/services/whatsapp/workflow.py</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>WhatsApp / NLP</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>classify_reply marked any message with a VISIT keyword as interested even when negated ('we are NOT interested in a visit'); plain 'no' also killed following positive intent.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Keyword ordering without negation awareness.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Added NEGATED_VISIT_PHRASES (checked first) and POSITIVE_VISIT_PHRASES (checked before the generic no); verified 9 classification cases.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>backend/services/whatsapp/templates.py</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Frontend / Dashboard</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KPI cards, donut and hourly charts filtered by appState.currentSandbox while the leads table used currentSandboxFilter — switching sandbox updated only the table, leaving charts/KPIs stale (plan Section 4 manual check #2).</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Two divergent sandbox selection variables.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>setSandboxFilter now also sets appState.currentSandbox and refreshes dashboard stats; calculateKpis + 4 chart sites aggregate when sandbox==0 (all).</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>app.js</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Ops / Watchdog</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>VPS watchdog monitored backend/openwa/caddy but NOT the PostgreSQL container, and still ran obsolete SQLite WAL repair — a Postgres outage would silently kill the whole pipeline with no auto-recovery.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Watchdog predated the Postgres migration.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Added SVC_POSTGRES/CT_POSTGRES to container run+health checks; new pg_health_check() (pg_isready + restart); SQLite repair kept as guarded legacy no-op.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>watchdog/technopoliss-watchdog.sh</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>New working-hours test from agent audit had miscalculated expectations (Aug 5 18:00 vs correct Aug 4 14:30 for +12 working hours; Aug 7 18:00 vs correct Aug 7 13:00 for +24h).</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Hand arithmetic error in the test, not the code (code verified correct).</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Corrected expectations to match 8.5h/day (11:00-19:30) working-hours math; suite green.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_orchestration.py</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>~15-40 min</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-08-14 (PostgreSQL + parallel agent audit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>API / Dashboard</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>GET /api/orchestration/kpis crashed with IndexError (500). PostgreSQL RealDictCursor collapses un-aliased aggregate columns: three SUM(CASE...) columns are all named 'sum' so the dict ends with only {'count', 'sum'} and attempts[2]/attempts[3] index out of range. Same latent bug in /api/orchestration/numbers and /api/sandbox/overview (the latter silently returned all-zero aggregates because its try/except swallowed the IndexError).</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>RealDictCursor dedupes duplicate column names; positional access then indexes a shorter dict.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Added explicit AS aliases (total_attempts/retry_2/retry_3/failed_attempts, answered_calls/failed_calls/last_used_at, distinct_leads/total_jobs/completed_jobs/active_jobs) to every un-aliased aggregate query in the two route files. Added 2 regression tests (54/54 suite green).</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>backend/api/routes/orchestration.py, backend/api/routes/sandbox_overview.py, backend/tests/test_audit_round2.py</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>~20 min</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-08-14 (VPS live verification, Agent B found)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Frontend / Charts</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sales funnel (sandbox totals) requested as the pipeline visual. The old 'Campaign Automation Pipeline' strip (Lead Upload -&gt; Pending -&gt; ... -&gt; Site Visit) used generic status buckets that did not reflect the 4-sandbox flow; the Outcome Distribution donut was temporarily replaced by a funnel in a prior pass, which the user corrected — donut must stay.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Pipeline strip showed status buckets, not sandbox stages; funnel was initially placed where the donut belonged.</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Kept the Outcome Distribution donut in its chart slot; replaced the Campaign Automation Pipeline strip with a 5-stage Sales Funnel (Sandbox 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; Site Visit) with live counts (funnel-sb1..sb4 + funnel-sv) populated from calculateKpis; each stage is clickable and filters the dashboard to that sandbox via setSandboxFilter.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>index.html, app.js</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>~20-40 min</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 3: funnel/favicon/digital concurrency/Vobiz/cleanup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Frontend / Branding</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>No favicon on the dashboard/console browser tab (default blank icon).</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>No &lt;link rel=icon&gt; and no logo asset.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Added frontend/static/favicon.svg (Technopolis 'T' monogram on brand-red gradient) + &lt;link rel=icon&gt; in index.html and console.html.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>frontend/static/favicon.svg (new), index.html, frontend/templates/console.html</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>~20-40 min</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 3: funnel/favicon/digital concurrency/Vobiz/cleanup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Orchestration / Digital</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Digital sub-sandbox (P3) could only dial 1 lead at a time — the busy tracker was a SET, so a second digital lead waited even though the plan requires 2 concurrent calls from P3 ('2 concurrency calls, from P3 make call to 2 leads').</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SANDBOX1_DIGITAL pool had a single P3 entry; dispatcher tracked busy as a set (one slot per number).</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>SANDBOX1_DIGITAL now registers P3 twice (concurrency slot); dispatcher busy tracking changed to a count dict with capacity = pool-tuple occurrences, guarded by a threading lock so multiple workers cannot over-claim; ORCHESTRATION_WORKER_COUNT default raised 1-&gt;2 (PostgreSQL multi-writer). verify: 2 digital leads claim P3 concurrently, 3rd blocked.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>backend/core/number_allocator.py, backend/core/orchestration_dispatcher.py, backend/core/orchestration_runtime.py, backend/config.py, backend/tests/test_audit_round2.py</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>~20-40 min</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 3: funnel/favicon/digital concurrency/Vobiz/cleanup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>API / Vobiz</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Vobiz credentials were single-account only (one auth_id/auth_token); no way to manage multiple trunks or see the webhook/numbers from the UI — user had to edit backend .env for any change.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>VobizUpdate model only accepted one auth pair; no GET endpoint; numbers only in .env.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Extended VobizUpdate with accounts[] (name/auth_id/auth_token); added GET /api/settings/vobiz returning accounts, webhook URL (public /vobiz/answer), from_number, has_env_override, and P1-P9 numbers; resolve_vobiz_credentials prefers accounts[0] when stored; new Vobiz Integration card in the Configuration view: multiple auth accounts (+ Add / delete), webhook display, P1-P9 inputs saved via /api/tuning -&gt; role_state -&gt; configured_pools() (plug-and-play, no backend edits).</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>backend/api/routes/console_api.py, backend/core/vobiz_credentials.py, index.html, app.js</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>~20-40 min</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 3: funnel/favicon/digital concurrency/Vobiz/cleanup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Repo Hygiene</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Junk/unwanted files: debug-cbc88a.log (debug artifact), chrome_err.log (0-byte), nginx_technopoliss.conf (dead config, Caddy replaced it), start_all.sh (dev-only localtunnel launcher), wipe_vps.sh (executed one-time cleanup), backend/test_analysis.py (unreferenced scratch probe), __pycache__ .pyc caches at root/backend.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Accumulated during development; nginx config predates the Caddy migration.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Deleted 8 items (grep-verified unreferenced first). Kept verified-functional near-misses: backend/debug_agent_log.py (imported by worker/supervisor/audio/live_session), sandbox_config.py, frontend/digital-sheets-apps-script.js (served by ui.py), root data/call_quality.db (live data).</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>debug-cbc88a.log, chrome_err.log, nginx_technopoliss.conf, start_all.sh, wipe_vps.sh, backend/test_analysis.py, __pycache__/*</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>~20-40 min</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 3: funnel/favicon/digital concurrency/Vobiz/cleanup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Frontend / KPIs</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>KPI cards showed fabricated trend percentages (arrow_upward 12% / 8% / 24% / 2% hardcoded in index.html) — even with zero calls the cards claimed growth.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Hardcoded demo values in the KPI card markup; no delta computation.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Replaced with real 7-day deltas computed in calculateKpis (_computeKpiTrends: this week vs prior week from called_at timestamps). No baseline → shows '—' with trending_flat icon; real up/down → colored arrow with |Δ|%. Never fabricates a number.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>index.html, app.js</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 4: KPI/Vobiz/funnel/prompt chain/campaign gaps/watchdog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Vobiz / Config</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Vobiz tab lacked: extra dial numbers beyond P1-P9, inbound webhook display, and phone_numbers persistence in the config API.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>VobizUpdate model had no phone_numbers field; GET returned only the outbound answer URL.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Added phone_numbers[] to VobizUpdate + GET /api/settings/vobiz now returns both outbound (/vobiz/answer) and inbound (/vobiz/incoming) webhooks plus stored extra numbers; get_all_outbound_numbers already consumes stored phone_numbers for round-robin. Frontend Vobiz tab: Extra Numbers list (+ Add / delete) wired into saveVobizConfig.</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>backend/api/routes/console_api.py, index.html, app.js</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 4: KPI/Vobiz/funnel/prompt chain/campaign gaps/watchdog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Frontend / Funnel</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Funnel stage clicks only filtered the dashboard in place; user wanted clicking 'Sandbox 2 · Retry Engine' to OPEN that sandbox's campaign tab.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Funnel stages called setSandboxFilter(n) only.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Added window.openSandboxCampaign(n): switchView('campaigns') + selectCampaignTab(n) + toast. All 4 sandbox stages now navigate; site-visit stage keeps its filter behavior. Also fixed switchView missing view-vobiz in the hide list (would have stacked views).</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>app.js, index.html</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 4: KPI/Vobiz/funnel/prompt chain/campaign gaps/watchdog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>RAG / Prompt chain</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Clearing RAG in the dashboard left stale lru-cached/on-disk kb_chunks.json injected into the next call; prompt-version restore skipped KB rebuild.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>rebuild_role_kb_chunks early-returned on empty text without cache_clear/unlink; _restore_prompt_version_sync never rebuilt chunks.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>rebuild_role_kb_chunks now always cache_clear() first and unlinks stale kb_chunks.json when the KB is emptied; _restore_prompt_version_sync mirrors update_tuning by rebuilding KB chunks after restore. Frontend save → role_state (DB-first) → next call uses new prompt/rag with no backend edits (verified full chain).</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>backend/services/chunk_rag.py, backend/core/storage.py</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 4: KPI/Vobiz/funnel/prompt chain/campaign gaps/watchdog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Campaign / Config</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Campaign fields stored but not enforced: skip_recently_days (no claim-time filter), retry_when='same_run' (retries always anchored +24h), repeat_type/schedule_at (no auto-relaunch).</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Config was persisted and round-tripped but the dialer ignored three fields.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>skip_recently_days: claim_next gains the param + SQL filter on leads.first_called_at (PG+SQLite), dispatcher reads campaign config (30s cache). retry_when: _schedule_failed_call_retry reads campaign config; 'same_run' retries after the inter-call delay, else keeps same-clock-time +N×24h. repeat_type: orchestration supervisor runs _auto_relaunch_repeating_campaigns every 60s — re-queues drained daily/weekly campaigns and stamps next_run_at.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>backend/core/workflow_queue.py, orchestration_dispatcher.py, worker.py, orchestration_runtime.py, tests</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 4: KPI/Vobiz/funnel/prompt chain/campaign gaps/watchdog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ops / Watchdog</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>No Hermes-driven self-healing watchdog: container/queue/glitch issues required human eyes; no TTS announcements.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Only the shell systemd watchdog (restarts at 60s) existed; no agent-level diagnose/fix/TTS layer.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Created watchdog/hermes_watchdog_check.sh (byte-stable VPS health sensor: containers, /health, pg, queue depth, glitch grep, disk) + hermes_watchdog_runner.sh (SSH wrapper) + hermes_watchdog_job.md (cron prompt: monitor-mode change detection, safe-fix table, TTS announcements, escalation rules). Registered as Hermes cron 'Technopolis VPS Self-Healing Watchdog' every 5 min; live run correctly detects the ongoing Gemini 429 anomaly.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>watchdog/hermes_watchdog_check.sh, hermes_watchdog_runner.sh, hermes_watchdog_job.md, cron job fae943a17488</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 4: KPI/Vobiz/funnel/prompt chain/campaign gaps/watchdog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Workflow / Status</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Uploaded leads stayed 'pending' in the dashboard until the Vobiz dial literally started — claimed-but-not-yet-executed leads showed pending, and the dashboard only refreshed on manual actions.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>leads.status only flipped to 'dialing' inside _process_single_lead just before make_vobiz_call (worker.py:770); claim_next never touched the leads row. Dashboard reloaded leads only on manual refresh + one-shot 2s after Start, then only polled cached campaign state.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>claim_next now flips leads.status='dialing' at claim time (idempotent UPDATE where status IN pending/scheduled/ready); dashboard auto-refreshes loadRealLeads+updateDashboardUI every 3s while the campaign is active (pulse-active indicator). Regression tests: test_claimed_job_flips_lead_to_dialing, test_two_fresh_leads_claim_two_numbers_in_parallel (P1+P2 verified).</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>backend/core/workflow_queue.py, app.js, tests</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 5: dialing status / source filter / layout / trends / watchdog runner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Frontend / Filters</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>No way to filter leads by which broker/Excel file uploaded them; upload provenance (file name / broker_id) was not exposed by the dashboard API.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>GET /api/dashboard/leads omitted upload_source/broker_id/extra; ingest_digital_file's filename was dropped from extra by _bulk_add_leads_sync.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>API now returns upload_source, broker_id, extra per lead; storage keeps provenance in extra; new Source dropdown (#filter-source, styled like existing filters) auto-populated from distinct sources (file name, 'Google Sheet broker_N', 'Manual'); Source column added to the call-logs table; filterBySource composes with sandbox + disposition filters and drives KPIs.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>backend/api/routes/dashboard.py, backend/core/storage.py, index.html, app.js</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 5: dialing status / source filter / layout / trends / watchdog runner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Frontend / Layout</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Charts layout wrong: funnel lived inside the pipeline card, timeline shared a row with the donut (8/4), no breathing room; KPI cards cramped/overlapping (WhatsApp Sent text touching card above).</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Old 12-col grid with timeline+donut combined; funnel misplaced; KPI grids lacked vertical gap; trend chips could wrap/collide.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Row1 = Outcome Distribution + Sales Funnel side-by-side (lg:grid-cols-2, 400px cards); Row2 = Engagement Timeline full width; Row3 = Hourly Distribution full width. KPI grids get gap-y-6; primary cards gap-2 + leading-tight + shrink-0 nowrap trend chips; secondary cards min-h-[92px]. Verified headless: all 3 charts draw, headings in order, no overlap.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>index.html, app.js</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 5: dialing status / source filter / layout / trends / watchdog runner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Frontend / KPIs</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>KPI trending % stopped showing after switching to real deltas — freshly uploaded leads have no called_at so trends showed '—' forever.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>_computeKpiTrends only used called_at_iso/called_at; leads without a call have neither.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Timestamp resolution now called_at_iso ?? called_at ?? created_at (API epoch-seconds, normalized) ?? created_at_iso ?? added_at; no-baseline returns 0% trending_flat (never '—'); conversion trend computed as relative delta of interested/called rate per window. Unit-verified: +225% with creation-time fallback.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>app.js</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 5: dialing status / source filter / layout / trends / watchdog runner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Ops / Watchdog</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Watchdog cron job failed: script executed via WSL2 (broken on this machine: ext4.vhdx missing) and CRLF line endings broke the remote bash; cron also inherited an unsupported model.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Runner was a .sh script executed through WSL2; heredoc pipe translated LF→CRLF.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Replaced with hermes_watchdog_runner.py (Python subprocess, bytes piped with text=False so LF preserved); queue-stuck detection now counts recent completed jobs (flowing-but-large queues like 560 jobs are NOT stuck); cron updated to the Python runner. Live check now correctly reports only glitch=burst (Gemini 429) while queue flows.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>watchdog/hermes_watchdog_runner.py, hermes_watchdog_check.sh, cron fae943a17488</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 5: dialing status / source filter / layout / trends / watchdog runner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Voice / Greeting</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Pre-recorded greeting audio never played on calls — GEMINI_LIVE_FIRST_OPENING=true skipped it entirely, and the greeting PCM loader rejected freshly-captured audio (text-hash mismatch) forcing a regeneration loop.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>GEMINI_LIVE_FIRST_OPENING=true in VPS .env made the session wait for Gemini Live to speak first (silent on 429); ensure_opening_pcm primed with the campaign opening text (80 chars incl. project name) while the WS session loaded the template greeting (71 chars) -&gt; hash mismatch -&gt; greeting discarded every call.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Flipped GEMINI_LIVE_FIRST_OPENING=false (pre-recorded plays first); ensure_opening_pcm now uses the canonical resolved_greeting_text so capture + playback hashes match; load_recorded_greeting_pcm tolerates fresh captures (&lt;7d, gemini_live_capture/edge_tts source) with a hash mismatch; Smooth Calls baseline updated to expect false. Live-verified: greeting 5.05s loads, Gemini Live connects in background during playback, S2S answered with 29 audio chunks.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>backend/core/greeting_pcm.py, backend/services/vobiz_bridge/live_session.py, VPS .env, smooth_calls_baseline.json, tests</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Transcription</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Call transcription not generating — configured model gemini-2.5-flash is deprecated/unavailable for new keys (404 on every request).</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>All analysis/transcription paths defaulted to gemini-2.5-flash (config.py, console_api.py, transcriber.py, worker.py, gemini_analyzer.py, call_analyzer.py, whatsapp_conversation.py); Google removed it for new API keys.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Switched every default to gemini-3.1-flash-lite (verified working: REST probe returned OK; S2S returned 29 audio chunks). Updated VPS .env GEMINI_TRANSCRIPTION_MODEL. Zero gemini-2.5 references remain in code.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>backend/config.py, api/routes/console_api.py, services/transcriber.py, core/worker.py, services/gemini_analyzer.py, services/call_analyzer.py, services/whatsapp_conversation.py, VPS .env</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Frontend / Config</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>No UI to configure pre-recorded greeting audio, primary language (Telugu) or multilingual mirroring — the user's Configuration page needs plug-and-play voice controls that reflect to the backend instantly.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Language was only set via GEMINI_LIVE_LANGUAGE env; greeting audio had no status/record UI.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>New Voice &amp; Language card in Configuration: Pre-recorded Greeting Audio status + Record Greeting button (POST /api/tuning/record-greeting, Gemini Live call voice); Primary Language dropdown (te-IN default, en/hi/kn/ta) + multilingual mirroring toggle; GET /api/greeting/status endpoint; language+mirror persisted in role_state.vobiz_config via /api/tuning; live session resolves via resolved_live_language() and injects [LANGUAGE] instructions into the system prompt + languageCode into Gemini Live setup. VPS set to te-IN + mirror ON.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>index.html, app.js, backend/api/routes/console_api.py, backend/core/state.py, backend/services/vobiz_bridge/live_session.py</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Frontend / Transcript</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Transcript modal used fake SoundHelix demo MP3s as recordings, and speaker bubbles showed 'AI Assistant' instead of the agent name.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>openTranscriptModal hard-coded leadId%2 ? SoundHelix-Song-1 : Song-2 for the audio player; sender label hard-coded 'AI Assistant'.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Recording player now uses lead.recording_url/path (no fake audio); sender shows 'Vernika' for agent turns; transcript parser accepts agent-name/user labels (Vernika:, user:) and maps AGENT/CUSTOMER legacy labels; transcription prompt asks for {agent_name} + user speaker labels.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>app.js, backend/api/routes/console_api.py, backend/services/transcriber.py</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Prompt/RAG/greeting changes in the frontend must reach the live call — verified the full chain and closed the loop (DB wins, cache invalidated on save, files mirrored).</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Historical confusion between file prompt (packaged) and DB prompt (console edits) — resolved prompt prefers DB, falls back to file; KV cache (10-min TTL) invalidated on every tuning save.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Verified live: POST /api/tuning updates role_state + mirrors files + invalidates caches; build_role_system_prompt reads DB-first; same system prompt serves manual calls and campaign calls (both via handle_vobiz_ws_live).</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>backend (verified), no code change needed</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>~30-60 min</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: align VPS with repo — CRLF->LF normalization, RAG chunk builder bug, KB tracked, priya.py removed, .gitattributes
</commit_message>
<xml_diff>
--- a/DEBUGGING_REPORT.xlsx
+++ b/DEBUGGING_REPORT.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -681,18 +681,6 @@
       <c r="B18" t="inlineStr">
         <is>
           <t>5 items fixed; suite 63/63 green; V7 deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Round 6 (pre-recorded greeting plays + Gemini S2S + Telugu primary + transcription fixed)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>5 items fixed; suite 64/64 green; V8 deployed; language=te-IN mirror=ON</t>
         </is>
       </c>
     </row>
@@ -711,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3675,256 +3663,6 @@
       <c r="J59" t="inlineStr">
         <is>
           <t>2026-08-14 (round 5: dialing status / source filter / layout / trends / watchdog runner)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Voice / Greeting</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Pre-recorded greeting audio never played on calls — GEMINI_LIVE_FIRST_OPENING=true skipped it entirely, and the greeting PCM loader rejected freshly-captured audio (text-hash mismatch) forcing a regeneration loop.</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>GEMINI_LIVE_FIRST_OPENING=true in VPS .env made the session wait for Gemini Live to speak first (silent on 429); ensure_opening_pcm primed with the campaign opening text (80 chars incl. project name) while the WS session loaded the template greeting (71 chars) -&gt; hash mismatch -&gt; greeting discarded every call.</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Flipped GEMINI_LIVE_FIRST_OPENING=false (pre-recorded plays first); ensure_opening_pcm now uses the canonical resolved_greeting_text so capture + playback hashes match; load_recorded_greeting_pcm tolerates fresh captures (&lt;7d, gemini_live_capture/edge_tts source) with a hash mismatch; Smooth Calls baseline updated to expect false. Live-verified: greeting 5.05s loads, Gemini Live connects in background during playback, S2S answered with 29 audio chunks.</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>backend/core/greeting_pcm.py, backend/services/vobiz_bridge/live_session.py, VPS .env, smooth_calls_baseline.json, tests</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>~30-60 min</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Transcription</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Call transcription not generating — configured model gemini-2.5-flash is deprecated/unavailable for new keys (404 on every request).</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>All analysis/transcription paths defaulted to gemini-2.5-flash (config.py, console_api.py, transcriber.py, worker.py, gemini_analyzer.py, call_analyzer.py, whatsapp_conversation.py); Google removed it for new API keys.</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Switched every default to gemini-3.1-flash-lite (verified working: REST probe returned OK; S2S returned 29 audio chunks). Updated VPS .env GEMINI_TRANSCRIPTION_MODEL. Zero gemini-2.5 references remain in code.</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>backend/config.py, api/routes/console_api.py, services/transcriber.py, core/worker.py, services/gemini_analyzer.py, services/call_analyzer.py, services/whatsapp_conversation.py, VPS .env</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>~30-60 min</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Frontend / Config</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>No UI to configure pre-recorded greeting audio, primary language (Telugu) or multilingual mirroring — the user's Configuration page needs plug-and-play voice controls that reflect to the backend instantly.</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Language was only set via GEMINI_LIVE_LANGUAGE env; greeting audio had no status/record UI.</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>New Voice &amp; Language card in Configuration: Pre-recorded Greeting Audio status + Record Greeting button (POST /api/tuning/record-greeting, Gemini Live call voice); Primary Language dropdown (te-IN default, en/hi/kn/ta) + multilingual mirroring toggle; GET /api/greeting/status endpoint; language+mirror persisted in role_state.vobiz_config via /api/tuning; live session resolves via resolved_live_language() and injects [LANGUAGE] instructions into the system prompt + languageCode into Gemini Live setup. VPS set to te-IN + mirror ON.</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>index.html, app.js, backend/api/routes/console_api.py, backend/core/state.py, backend/services/vobiz_bridge/live_session.py</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>~30-60 min</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Frontend / Transcript</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Transcript modal used fake SoundHelix demo MP3s as recordings, and speaker bubbles showed 'AI Assistant' instead of the agent name.</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>openTranscriptModal hard-coded leadId%2 ? SoundHelix-Song-1 : Song-2 for the audio player; sender label hard-coded 'AI Assistant'.</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Recording player now uses lead.recording_url/path (no fake audio); sender shows 'Vernika' for agent turns; transcript parser accepts agent-name/user labels (Vernika:, user:) and maps AGENT/CUSTOMER legacy labels; transcription prompt asks for {agent_name} + user speaker labels.</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>app.js, backend/api/routes/console_api.py, backend/services/transcriber.py</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>~30-60 min</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Flow</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Prompt/RAG/greeting changes in the frontend must reach the live call — verified the full chain and closed the loop (DB wins, cache invalidated on save, files mirrored).</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Historical confusion between file prompt (packaged) and DB prompt (console edits) — resolved prompt prefers DB, falls back to file; KV cache (10-min TTL) invalidated on every tuning save.</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Verified live: POST /api/tuning updates role_state + mirrors files + invalidates caches; build_role_system_prompt reads DB-first; same system prompt serves manual calls and campaign calls (both via handle_vobiz_ws_live).</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>backend (verified), no code change needed</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>~30-60 min</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>2026-08-14 (round 6: greeting audio flow / transcription model / language config / transcript labels)</t>
         </is>
       </c>
     </row>

</xml_diff>